<commit_message>
Actualizacao dos dados dos exercicios
</commit_message>
<xml_diff>
--- a/PAM_VERDE_2026_Baseline.xlsx
+++ b/PAM_VERDE_2026_Baseline.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -28672,6 +28672,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
@@ -28680,15 +28689,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -28927,6 +28927,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D6439EC-2526-4ED2-8778-ED43E26DD9C0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2D9617B4-6C84-4D7A-8C1E-C3670E7360B9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -28937,14 +28945,21 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D6439EC-2526-4ED2-8778-ED43E26DD9C0}">
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5E695D4-E1C0-4112-9B16-228E49F56615}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5E695D4-E1C0-4112-9B16-228E49F56615}"/>
 </file>
</xml_diff>